<commit_message>
inital commit for C16A-2
</commit_message>
<xml_diff>
--- a/data/ClueLayoutAdjTests.xlsx
+++ b/data/ClueLayoutAdjTests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\eclipse-workspace\C16A\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1591AFE0-8D5B-4F5A-8487-64507B708CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22970BCD-0521-4629-8FED-985FE00B3C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="1650" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>